<commit_message>
Phone: progress 1 in nyheder.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/nyheder.xlsx
+++ b/12-06-2026-vokab/nyheder.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -553,16 +553,16 @@
         <v>2026-06-18</v>
       </c>
       <c r="S2" t="str">
+        <v>0</v>
+      </c>
+      <c r="T2" t="str">
+        <v>2.1</v>
+      </c>
+      <c r="U2" t="str">
+        <v>0</v>
+      </c>
+      <c r="V2" t="str">
         <v>1</v>
-      </c>
-      <c r="T2" t="str">
-        <v>2.3</v>
-      </c>
-      <c r="U2" t="str">
-        <v>1</v>
-      </c>
-      <c r="V2" t="str">
-        <v>0</v>
       </c>
       <c r="W2" t="str">
         <v/>

</xml_diff>